<commit_message>
Reconcile PSI ledger UVA source identity
</commit_message>
<xml_diff>
--- a/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
+++ b/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0f951e2e94314ab6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="Rac5ad973ae6f4e1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rc848d663f8e94cc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="Rab3016530b9e415b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="R0b946f8d4380465b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="R04805c3b5e314b48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="Rfae70dde79f14837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R65c7dcb690d24342"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="Ra0e914da1cf44ddc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Ra51327b360da4273"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="R0c3c326448ad44cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="Reaf437570b1d412f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="Rd5034bbcbdba42fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="R7759bc869fd9433e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2600,7 +2600,7 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="31" t="str">
-        <x:v>WORK-343-UVA-CHILDREN-PL</x:v>
+        <x:v>UVA-DOPS-CHILDREN</x:v>
       </x:c>
       <x:c r="B42" s="31" t="str">
         <x:v>REI</x:v>
@@ -3287,20 +3287,20 @@
         <x:v>M343-008</x:v>
       </x:c>
       <x:c r="B19" s="21" t="str">
-        <x:v>WORK-343-UVA-CHILDREN-PL</x:v>
+        <x:v>UVA-DOPS-CHILDREN</x:v>
       </x:c>
       <x:c r="C19" s="21" t="str">
         <x:v>INSTITUTIONAL_OVERVIEW</x:v>
       </x:c>
       <x:c r="D19" s="21" t="str">
-        <x:v>NEW_SOURCE_CANDIDATE</x:v>
+        <x:v>EXISTING_GOVERNED_RECORD</x:v>
       </x:c>
       <x:c r="E19" s="21" t="str"/>
       <x:c r="F19" s="21" t="str">
         <x:v>https://med.virginia.edu/perceptual-studies/our-research/children-who-report-memories-of-previous-lives/</x:v>
       </x:c>
       <x:c r="G19" s="21" t="str">
-        <x:v>Ryan Hammons claim set unresolved</x:v>
+        <x:v>Reuse governed source UVA-DOPS-CHILDREN; Ryan Hammons claim set unresolved</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -4499,7 +4499,7 @@
         <x:v>Current source set</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>GitHub issues #343, #350 and #354; PR #352 corrected head a15878a; repository file interbrain-telepathy-mayim-bialik-source-crawl-v0.1.json; live verification of BIO-PK-001 bibliographic record.</x:v>
+        <x:v>GitHub issues #343, #350 and #354; PR #352 merged corrected head 6fa7415b08bf904268f9132560009021a0d468ee; repository file interbrain-telepathy-mayim-bialik-source-crawl-v0.1.json; live verification of BIO-PK-001 bibliographic record.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">

</xml_diff>

<commit_message>
fix(psi): preserve governed source identities
</commit_message>
<xml_diff>
--- a/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
+++ b/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R65c7dcb690d24342"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="Ra0e914da1cf44ddc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Ra51327b360da4273"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="R0c3c326448ad44cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="Reaf437570b1d412f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="Rd5034bbcbdba42fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="R7759bc869fd9433e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R147c1dd1c1e942f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="R6e570a377422401b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R0acb272f96f247f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="R23388698b16e4097"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="R073e6cbe36da46d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="Rbcbd2f839ee342a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="Re0c04f4f186048e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2223,7 +2223,7 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="21" t="str">
-        <x:v>COUNTER-TTG-2026</x:v>
+        <x:v>COUNTER-TTG-TELEPATHY-TAPES-2026-02-09</x:v>
       </x:c>
       <x:c r="B31" s="21" t="str">
         <x:v>TEL-007</x:v>
@@ -2324,7 +2324,7 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="31" t="str">
-        <x:v>MILTON-WISEMAN-1999</x:v>
+        <x:v>MILTON-WISEMAN-1999-GANZFELD</x:v>
       </x:c>
       <x:c r="B34" s="31" t="str">
         <x:v>TEL</x:v>
@@ -2359,7 +2359,7 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="21" t="str">
-        <x:v>GRAFF-RADFORD-2017</x:v>
+        <x:v>GRAFF-RADFORD-2017-CAUDATE-NETWORKS</x:v>
       </x:c>
       <x:c r="B35" s="21" t="str">
         <x:v>TEL-003</x:v>

</xml_diff>

<commit_message>
fix(psi): preserve PR 352 work identities
</commit_message>
<xml_diff>
--- a/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
+++ b/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R147c1dd1c1e942f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="R6e570a377422401b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R0acb272f96f247f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="R23388698b16e4097"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="R073e6cbe36da46d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="Rbcbd2f839ee342a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="Re0c04f4f186048e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2acb22db21e5430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="Rd90f0179121e4958"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R471b8949a91d4193"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="R2014719e9cca4d71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="R95652eee26c141f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="Rcaa3662a8fd64d77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="R32c5b419b03446c8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2394,7 +2394,7 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="31" t="str">
-        <x:v>WORK-343-SURVIVING-DEATH-2021</x:v>
+        <x:v>WORK-343-SURVIVING-DEATH-SERIES-2021</x:v>
       </x:c>
       <x:c r="B36" s="31" t="str">
         <x:v>NDE / MED / ADC / REI</x:v>
@@ -2427,7 +2427,7 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="21" t="str">
-        <x:v>WORK-343-UVA-COMPANION</x:v>
+        <x:v>WORK-343-UVA-SURVIVING-DEATH-COMPANION</x:v>
       </x:c>
       <x:c r="B37" s="21" t="str">
         <x:v>NDE / REI</x:v>
@@ -2495,7 +2495,7 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="21" t="str">
-        <x:v>WORK-343-SUDDUTH-2022</x:v>
+        <x:v>WORK-343-SUDDUTH-LEININGER-2022</x:v>
       </x:c>
       <x:c r="B39" s="21" t="str">
         <x:v>REI</x:v>
@@ -2565,7 +2565,7 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="21" t="str">
-        <x:v>WORK-343-SUDDUTH-REPLY-2022</x:v>
+        <x:v>WORK-343-SUDDUTH-RESPONSE-TO-TUCKER-2022</x:v>
       </x:c>
       <x:c r="B41" s="21" t="str">
         <x:v>REI</x:v>
@@ -2668,7 +2668,7 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="31" t="str">
-        <x:v>WORK-343-KAMP-2020</x:v>
+        <x:v>WORK-343-KAMP-BEREAVEMENT-2020</x:v>
       </x:c>
       <x:c r="B44" s="31" t="str">
         <x:v>ADC / BEREAVEMENT</x:v>
@@ -2703,7 +2703,7 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="21" t="str">
-        <x:v>WORK-343-SABUCEDO-2020</x:v>
+        <x:v>WORK-343-SABUCEDO-CULTURAL-BEREAVEMENT-2020</x:v>
       </x:c>
       <x:c r="B45" s="21" t="str">
         <x:v>ADC / BEREAVEMENT</x:v>
@@ -3140,7 +3140,7 @@
         <x:v>M343-001</x:v>
       </x:c>
       <x:c r="B12" s="31" t="str">
-        <x:v>WORK-343-SURVIVING-DEATH-2021</x:v>
+        <x:v>WORK-343-SURVIVING-DEATH-SERIES-2021</x:v>
       </x:c>
       <x:c r="C12" s="31" t="str">
         <x:v>OFFICIAL_CATALOGUE</x:v>
@@ -3161,7 +3161,7 @@
         <x:v>M343-002</x:v>
       </x:c>
       <x:c r="B13" s="21" t="str">
-        <x:v>WORK-343-UVA-COMPANION</x:v>
+        <x:v>WORK-343-UVA-SURVIVING-DEATH-COMPANION</x:v>
       </x:c>
       <x:c r="C13" s="21" t="str">
         <x:v>INSTITUTIONAL_COMPANION</x:v>
@@ -3224,7 +3224,7 @@
         <x:v>M343-005</x:v>
       </x:c>
       <x:c r="B16" s="31" t="str">
-        <x:v>WORK-343-SUDDUTH-2022</x:v>
+        <x:v>WORK-343-SUDDUTH-LEININGER-2022</x:v>
       </x:c>
       <x:c r="C16" s="31" t="str">
         <x:v>JOURNAL_RECORD</x:v>
@@ -3245,7 +3245,7 @@
         <x:v>M343-006</x:v>
       </x:c>
       <x:c r="B17" s="21" t="str">
-        <x:v>WORK-343-SUDDUTH-2022</x:v>
+        <x:v>WORK-343-SUDDUTH-LEININGER-2022</x:v>
       </x:c>
       <x:c r="C17" s="21" t="str">
         <x:v>AUTHOR_COMMENTARY</x:v>
@@ -3350,7 +3350,7 @@
         <x:v>M343-011</x:v>
       </x:c>
       <x:c r="B22" s="31" t="str">
-        <x:v>WORK-343-KAMP-2020</x:v>
+        <x:v>WORK-343-KAMP-BEREAVEMENT-2020</x:v>
       </x:c>
       <x:c r="C22" s="31" t="str">
         <x:v>INSTITUTIONAL_REPOSITORY</x:v>
@@ -3371,7 +3371,7 @@
         <x:v>M343-012</x:v>
       </x:c>
       <x:c r="B23" s="21" t="str">
-        <x:v>WORK-343-KAMP-2020</x:v>
+        <x:v>WORK-343-KAMP-BEREAVEMENT-2020</x:v>
       </x:c>
       <x:c r="C23" s="21" t="str">
         <x:v>FULL_TEXT_REPOSITORY</x:v>
@@ -3392,7 +3392,7 @@
         <x:v>M343-013</x:v>
       </x:c>
       <x:c r="B24" s="31" t="str">
-        <x:v>WORK-343-SABUCEDO-2020</x:v>
+        <x:v>WORK-343-SABUCEDO-CULTURAL-BEREAVEMENT-2020</x:v>
       </x:c>
       <x:c r="C24" s="31" t="str">
         <x:v>FULL_TEXT_REPOSITORY</x:v>
@@ -3687,7 +3687,7 @@
         <x:v>M343-026</x:v>
       </x:c>
       <x:c r="B37" s="21" t="str">
-        <x:v>WORK-343-SUDDUTH-REPLY-2022</x:v>
+        <x:v>WORK-343-SUDDUTH-RESPONSE-TO-TUCKER-2022</x:v>
       </x:c>
       <x:c r="C37" s="21" t="str">
         <x:v>JOURNAL_RECORD</x:v>

</xml_diff>

<commit_message>
fix(psi): preserve blog and episode manifestations
</commit_message>
<xml_diff>
--- a/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
+++ b/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2acb22db21e5430b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="Rd90f0179121e4958"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R471b8949a91d4193"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="R2014719e9cca4d71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="R95652eee26c141f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="Rcaa3662a8fd64d77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="R32c5b419b03446c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R86c2dcd63dfa4cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="Rd4338fe47b024d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rb7bde21d4b824c44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="R81a84b7b5f704ff4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="Rec1a2cfaafe74e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="Re82446f4a5814b4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="R544956b17f7f4e5c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -470,7 +470,7 @@
       </x:c>
       <x:c r="B6" t="n">
         <x:f>COUNTA(Sources!A2:A300)</x:f>
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -479,7 +479,7 @@
       </x:c>
       <x:c r="B7" t="n">
         <x:f>COUNTA(Manifestations!A2:A300)</x:f>
-        <x:v>36</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -497,7 +497,7 @@
       </x:c>
       <x:c r="B9" t="n">
         <x:f>COUNTIF(Sources!I2:I300,"REVIEW_REQUIRED")+COUNTIF(Sources!I2:I300,"REVIEW_CANDIDATE")</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2868,6 +2868,39 @@
         <x:v>Repository manifest</x:v>
       </x:c>
     </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>WORK-343-SUDDUTH-BLOG-LEININGER-2021</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>REI</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Michael Sudduth</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>Crash and Burn: James Leininger Story Debunked</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>AUTHOR_COMMENTARY</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>Counter-source</x:v>
+      </x:c>
+      <x:c r="G50"/>
+      <x:c r="H50" t="str">
+        <x:v>https://michaelsudduth.com/crash-and-burn-james-leininger-story-debunked/</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>REVIEW_REQUIRED</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>Author commentary related to the journal critique; derivative in evidential lineage and not an independent replication</x:v>
+      </x:c>
+      <x:c r="K50" t="str">
+        <x:v>Issue #343 / PR #352</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3245,7 +3278,7 @@
         <x:v>M343-006</x:v>
       </x:c>
       <x:c r="B17" s="21" t="str">
-        <x:v>WORK-343-SUDDUTH-LEININGER-2022</x:v>
+        <x:v>WORK-343-SUDDUTH-BLOG-LEININGER-2021</x:v>
       </x:c>
       <x:c r="C17" s="21" t="str">
         <x:v>AUTHOR_COMMENTARY</x:v>
@@ -3258,7 +3291,7 @@
         <x:v>https://michaelsudduth.com/crash-and-burn-james-leininger-story-debunked/</x:v>
       </x:c>
       <x:c r="G17" s="21" t="str">
-        <x:v>Not independent of critique lineage</x:v>
+        <x:v>Author commentary related to the journal critique; derivative in evidential lineage and not an independent replication</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -3701,6 +3734,69 @@
       </x:c>
       <x:c r="G37" s="21" t="str">
         <x:v>Discovered chain-gap reply</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>M-MBB-CHARLES-LIU-2026-09-02-WATCH</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>MBB-CHARLES-LIU-2026-09-02</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>OFFICIAL_WATCH_PAGE</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>ALTERNATE_MANIFESTATION</x:v>
+      </x:c>
+      <x:c r="E38"/>
+      <x:c r="F38" t="str">
+        <x:v>https://www.bialikbreakdown.com/watch-podcast/near-death-experiences-telepathy-the-multiverse-an-astrophysicist-explains-dr-charles-liu</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>Alternate governed episode URL; same podcast record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>M-MBB-SHARON-STONE-2026-09-09-PART2</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>MBB-SHARON-STONE-2026-09-08-09</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>OFFICIAL_EPISODE_PAGE</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>ALTERNATE_MANIFESTATION</x:v>
+      </x:c>
+      <x:c r="E39"/>
+      <x:c r="F39" t="str">
+        <x:v>https://www.bialikbreakdown.com/episodes/part-two-sharon-stone-saw-the-afterlife-5-orbs-told-her-to-stay-share-their-message</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>Part Two URL; same multipart podcast record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>M-MBB-LISA-KUDROW-2026-07-23-PART2</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>MBB-LISA-KUDROW-2026-07-21-23</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>OFFICIAL_EPISODE_PAGE</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>ALTERNATE_MANIFESTATION</x:v>
+      </x:c>
+      <x:c r="E40"/>
+      <x:c r="F40" t="str">
+        <x:v>https://www.bialikbreakdown.com/episodes/part-two-psychic-ability-energy-healing-remote-viewing-her-100-success-rate-lisa-kudrow</x:v>
+      </x:c>
+      <x:c r="G40" t="str">
+        <x:v>Part Two URL; same multipart podcast record</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(psi): preserve podcast catalog manifestation
</commit_message>
<xml_diff>
--- a/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
+++ b/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R86c2dcd63dfa4cf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="Rd4338fe47b024d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rb7bde21d4b824c44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="R81a84b7b5f704ff4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="Rec1a2cfaafe74e4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="Re82446f4a5814b4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="R544956b17f7f4e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1070f7301b2049f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="2" r:id="Rced3c4888dd2462e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Re95763371ce444ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifestations" sheetId="4" r:id="Rbcc489d295494671"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="5" r:id="Rbb8d74d393994c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 001 · BIO-PK" sheetId="6" r:id="R2e59381be7574c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" r:id="R24f2b683991a4f6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -479,7 +479,7 @@
       </x:c>
       <x:c r="B7" t="n">
         <x:f>COUNTA(Manifestations!A2:A300)</x:f>
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -3799,6 +3799,27 @@
         <x:v>Part Two URL; same multipart podcast record</x:v>
       </x:c>
     </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>M-MBB-KY-DICKENS-2025-10-24-CATALOG</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>MBB-KY-DICKENS-2025-10-24</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>CORROBORATING_PODCAST_CATALOG</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>ALTERNATE_MANIFESTATION</x:v>
+      </x:c>
+      <x:c r="E41"/>
+      <x:c r="F41" t="str">
+        <x:v>https://thetelepathytapes.com/podcast/</x:v>
+      </x:c>
+      <x:c r="G41" t="str">
+        <x:v>Corroborating governed catalog URL; same podcast source lineage</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(psi): add verified Radin 2008 publication locator
Fill the existing RADIN-2008-DI DOI and primary URL cells using DOI 10.1016/j.explore.2008.04.002 and PubMed 18602616. Refresh workbook integrity fields only.

Preserve 8 packets, 49 sources, 40 manifestations, HOLD dispositions and every closed governance gate.
</commit_message>
<xml_diff>
--- a/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
+++ b/references/psi/AkashicNET_PSI_Master_Ledger_2026-09-17.xlsx
@@ -1698,8 +1698,12 @@
       <x:c r="F15" s="21" t="str">
         <x:v>Physiological correlation</x:v>
       </x:c>
-      <x:c r="G15" s="21" t="str"/>
-      <x:c r="H15" s="21" t="str"/>
+      <x:c r="G15" s="21" t="str">
+        <x:v>10.1016/j.explore.2008.04.002</x:v>
+      </x:c>
+      <x:c r="H15" s="21" t="str">
+        <x:v>https://pubmed.ncbi.nlm.nih.gov/18602616/</x:v>
+      </x:c>
       <x:c r="I15" s="33" t="str">
         <x:v>HOLD</x:v>
       </x:c>

</xml_diff>